<commit_message>
use tasks to get fields
</commit_message>
<xml_diff>
--- a/services/ami/ami/ami_weekly_status_report/per_project/Huckleberry/Huckleberry_wsr_template.xlsx
+++ b/services/ami/ami/ami_weekly_status_report/per_project/Huckleberry/Huckleberry_wsr_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId2"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="127">
   <si>
     <t xml:space="preserve">Huckleberry VFX Vendor Weekly Report </t>
   </si>
@@ -339,31 +339,111 @@
     <t xml:space="preserve">{sg_turnover_date}</t>
   </si>
   <si>
-    <t xml:space="preserve">{layout_sg_blocking}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{layout_due_date}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{animation_sg_blocking}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{animation_due_date}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{fx_sg_blocking}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{fx_due_date}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{sg_comp_1st_pass_date}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{sg_comp_first_pass}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{sg_proposed_creative_final_date}</t>
+    <t xml:space="preserve">{layout___sg_blocking}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{layout___due_date}</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{animation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF067D17"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">___sg_blocking_date</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">}</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">{animation___due_date}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{fx___sg_blocking}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{fx___due_date}</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF067D17"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">compositing___sg_blocking_date</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">}</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF067D17"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">sg_wip_comp</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">}</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">{sg_pot_final_comp}</t>
   </si>
   <si>
     <t xml:space="preserve">{sg_final_due}</t>
@@ -430,7 +510,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -451,6 +531,32 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF067D17"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF067D17"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF067D17"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -501,7 +607,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -522,6 +628,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -531,6 +641,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF067D17"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -540,7 +710,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.31"/>
@@ -865,7 +1035,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:U4"/>
-  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.35"/>
@@ -874,11 +1044,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="17.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="23.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="17.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="19.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="32.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="22.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="16.64"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="19.81"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="24.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="19.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="39.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="34.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="31.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="16.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="22.48"/>
@@ -955,7 +1126,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -998,10 +1169,10 @@
       <c r="N3" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="O3" s="0" t="s">
+      <c r="O3" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="P3" s="0" t="s">
+      <c r="P3" s="5" t="s">
         <v>112</v>
       </c>
       <c r="Q3" s="0" t="s">
@@ -1042,7 +1213,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q4"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.08"/>
@@ -1108,9 +1279,7 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>4</v>
-      </c>
+      <c r="A3" s="3"/>
       <c r="B3" s="3" t="s">
         <v>98</v>
       </c>

</xml_diff>

<commit_message>
adding zed tasks and update hb wsr template
</commit_message>
<xml_diff>
--- a/services/ami/ami/ami_weekly_status_report/per_project/Huckleberry/Huckleberry_wsr_template.xlsx
+++ b/services/ami/ami/ami_weekly_status_report/per_project/Huckleberry/Huckleberry_wsr_template.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="134">
   <si>
     <t xml:space="preserve">Huckleberry VFX Vendor Weekly Report </t>
   </si>
@@ -503,9 +503,6 @@
     <t xml:space="preserve">{sg_asset_type}</t>
   </si>
   <si>
-    <t xml:space="preserve">{code}</t>
-  </si>
-  <si>
     <t xml:space="preserve">{sg_shared}</t>
   </si>
   <si>
@@ -535,7 +532,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -583,6 +580,11 @@
       <family val="3"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -626,7 +628,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -648,6 +650,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -729,7 +735,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.31"/>
@@ -1054,7 +1060,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:U4"/>
-  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.8046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.35"/>
@@ -1233,7 +1239,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q4"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.08"/>
@@ -1313,14 +1319,14 @@
       <c r="B3" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>127</v>
+      <c r="C3" s="6" t="s">
+        <v>99</v>
       </c>
       <c r="D3" s="0" t="s">
         <v>100</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F3" s="0" t="s">
         <v>102</v>
@@ -1329,29 +1335,29 @@
         <v>103</v>
       </c>
       <c r="H3" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="I3" s="0" t="s">
         <v>129</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="J3" s="0" t="s">
         <v>130</v>
       </c>
-      <c r="J3" s="0" t="s">
+      <c r="K3" s="0" t="s">
         <v>131</v>
-      </c>
-      <c r="K3" s="0" t="s">
-        <v>132</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>109</v>
       </c>
       <c r="M3" s="3"/>
       <c r="N3" s="0" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O3" s="0" t="s">
         <v>115</v>
       </c>
       <c r="P3" s="0" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Q3" s="3" t="s">
         <v>117</v>

</xml_diff>